<commit_message>
Matrice: coloanele 'Descriere Control (Criterii)' si 'Cadru de reglementare (Criterii)'; numele vechi acceptate in continuare; exemplu si README actualizate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Input/MatriceDeIntrodus.exemplu.xlsx
+++ b/Data/Input/MatriceDeIntrodus.exemplu.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,67 +417,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proces</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Arie</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>SubArie</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Descriere Risc</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tip Risc</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Denumire Control</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Descriere Control</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Descriere Control (Criterii)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tip Control</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Frecventa Control</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Cadru de reglementare Control</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Cadru de reglementare (Criterii)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Denumire Test</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Tehnici de Testare</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Detalii Tehnici de Testare</t>
         </is>

</xml_diff>

<commit_message>
Matrice: coloana 'Cod referinta APR (Nr. Crt.)' (prima), scrisa la fiecare test in campul CodApr de pe tab-ul Tehnici De Testare; matricele fara coloana raman valide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Input/MatriceDeIntrodus.exemplu.xlsx
+++ b/Data/Input/MatriceDeIntrodus.exemplu.xlsx
@@ -413,71 +413,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Cod referinta APR (Nr. Crt.)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Proces</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Arie</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>SubArie</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Descriere Risc</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tip Risc</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Denumire Control</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Descriere Control (Criterii)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tip Control</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Frecventa Control</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Cadru de reglementare (Criterii)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Denumire Test</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Tehnici de Testare</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Detalii Tehnici de Testare</t>
         </is>
@@ -486,61 +491,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Creditare</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Analiza creditului</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Evaluare incompleta a bonitatii</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Risc de credit</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Verificare dosar</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Descriere Verificare dosar</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Preventiv</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Lunar</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Regulament intern</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Test dosar 1</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Interviul; Examinarea</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Detalii Test dosar 1</t>
         </is>
@@ -549,61 +559,66 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Creditare</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Analiza creditului</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Evaluare incompleta a bonitatii</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Risc de credit</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Verificare dosar</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Descriere Verificare dosar</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Preventiv</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Lunar</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Regulament intern</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Test dosar 2</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Observarea</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Detalii Test dosar 2</t>
         </is>
@@ -612,65 +627,70 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Creditare</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Analiza creditului</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Persoane fizice</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Documente lipsa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Risc operational</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Checklist documente</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Descriere Checklist documente</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Preventiv</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Zilnic sau ori de cate ori este nevoie</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Regulament intern</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Test checklist</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Validarea; Recalcularea</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Detalii Test checklist</t>
         </is>
@@ -679,61 +699,66 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Creditare</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Aprobare</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Depasire competente</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Risc de conformitate</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Matrice competente</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Descriere Matrice competente</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Preventiv</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Trimestrial</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Regulament intern</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Test competente</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Examinarea</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Detalii Test competente</t>
         </is>

</xml_diff>

<commit_message>
Test: coloanele 'Auditor alocat' (bife in ResponsabilTest, potrivire toleranta a numelor, negasitele/ambiguele raportate in log + rezumat) si 'Termen finalizare test' (camp calendar, cu verificare)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Input/MatriceDeIntrodus.exemplu.xlsx
+++ b/Data/Input/MatriceDeIntrodus.exemplu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,16 @@
           <t>Detalii Tehnici de Testare</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Auditor alocat</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Termen finalizare test</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -555,6 +565,16 @@
           <t>Detalii Test dosar 1</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Popescu Ion; Ionescu Ana</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -623,6 +643,16 @@
           <t>Detalii Test dosar 2</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Popescu Ion; Ionescu Ana</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -695,6 +725,16 @@
           <t>Detalii Test checklist</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Popescu Ion; Ionescu Ana</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -761,6 +801,16 @@
       <c r="N5" t="inlineStr">
         <is>
           <t>Detalii Test competente</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Popescu Ion; Ionescu Ana</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>